<commit_message>
Added shortcuts for mouse
</commit_message>
<xml_diff>
--- a/host-scripts/screen_resolutions.xlsx
+++ b/host-scripts/screen_resolutions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raul.mzabala\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raul.mzabala\Local data\macropad_automator\host-scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD726B84-6465-4137-8F8D-11D7FD2D9E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399AB9A8-7D56-4365-A056-BC0A70ABAC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{F25BA907-62E5-4DE0-803B-72E5CA0E679E}"/>
+    <workbookView xWindow="2370" yWindow="-14610" windowWidth="21600" windowHeight="11700" xr2:uid="{F25BA907-62E5-4DE0-803B-72E5CA0E679E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Ratio</t>
   </si>
@@ -48,6 +48,15 @@
   </si>
   <si>
     <t>%</t>
+  </si>
+  <si>
+    <t>Vert</t>
+  </si>
+  <si>
+    <t>Hor2</t>
+  </si>
+  <si>
+    <t>Match</t>
   </si>
 </sst>
 </file>
@@ -99,7 +108,23 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="13" formatCode="0%"/>
     </dxf>
@@ -146,7 +171,7 @@
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>333690</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>67273</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -184,16 +209,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74F3B700-FB14-47FB-BBF5-EB81842DF844}" name="Table1" displayName="Table1" ref="G8:J20" totalsRowShown="0">
-  <autoFilter ref="G8:J20" xr:uid="{74F3B700-FB14-47FB-BBF5-EB81842DF844}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74F3B700-FB14-47FB-BBF5-EB81842DF844}" name="Table1" displayName="Table1" ref="G8:M20" totalsRowShown="0">
+  <autoFilter ref="G8:M20" xr:uid="{74F3B700-FB14-47FB-BBF5-EB81842DF844}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="TRUE"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C0824456-FD14-405A-88BA-F1A4599EED07}" name="Hor"/>
     <tableColumn id="2" xr3:uid="{62BFAFFA-A16A-418F-80BA-0766D7E71056}" name="Ver"/>
-    <tableColumn id="3" xr3:uid="{E1B9CFE3-A891-4260-B46C-58A49AE8B4FB}" name="Ratio" dataDxfId="1" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{E1B9CFE3-A891-4260-B46C-58A49AE8B4FB}" name="Ratio" dataDxfId="5" dataCellStyle="Percent">
       <calculatedColumnFormula>G9/H9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B91E335B-2807-4521-9854-46F0EDAEDAC2}" name="%" dataDxfId="0" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{B91E335B-2807-4521-9854-46F0EDAEDAC2}" name="%" dataDxfId="4" dataCellStyle="Percent">
       <calculatedColumnFormula>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{326C0564-3986-45C8-AF40-8E81A5AE3EDD}" name="Vert" dataDxfId="3">
+      <calculatedColumnFormula>Table1[[#This Row],[Hor]]/$G$9</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{23F9BB6F-D88A-4E1E-A105-C52B456ABB76}" name="Hor2" dataDxfId="2">
+      <calculatedColumnFormula>Table1[[#This Row],[Ver]]/$H$9</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{627D3C5F-846E-4F63-B5F1-03FF778FD2F0}" name="Match" dataDxfId="1">
+      <calculatedColumnFormula>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -517,10 +557,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{167FCC48-857D-4038-80CF-8DE97A674B4A}">
-  <dimension ref="G8:O20"/>
+  <dimension ref="G8:P20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="8" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G8" t="s">
         <v>1</v>
       </c>
@@ -533,8 +573,17 @@
       <c r="J8" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="K8" t="s">
+        <v>4</v>
+      </c>
+      <c r="L8" t="s">
+        <v>5</v>
+      </c>
+      <c r="M8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G9">
         <v>2560</v>
       </c>
@@ -549,18 +598,30 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>1</v>
       </c>
-      <c r="M9">
+      <c r="K9">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>1</v>
+      </c>
+      <c r="M9" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>1</v>
+      </c>
+      <c r="N9">
         <v>1920</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>1080</v>
       </c>
-      <c r="O9">
-        <f>M9/N9</f>
+      <c r="P9">
+        <f>N9/O9</f>
         <v>1.7777777777777777</v>
       </c>
     </row>
-    <row r="10" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G10">
         <v>2048</v>
       </c>
@@ -575,15 +636,27 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.76800000000000002</v>
       </c>
-      <c r="M10">
-        <f>O9*N10</f>
+      <c r="K10">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.8</v>
+      </c>
+      <c r="L10">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.96</v>
+      </c>
+      <c r="M10" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <f>P9*O10</f>
         <v>2560</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>1440</v>
       </c>
     </row>
-    <row r="11" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G11">
         <v>1920</v>
       </c>
@@ -598,12 +671,24 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.5625</v>
       </c>
-      <c r="M11">
-        <f>M10-860-860</f>
+      <c r="K11">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.75</v>
+      </c>
+      <c r="L11">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.75</v>
+      </c>
+      <c r="M11" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <f>N10-860-860</f>
         <v>840</v>
       </c>
     </row>
-    <row r="12" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G12">
         <v>1920</v>
       </c>
@@ -618,8 +703,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.50624999999999998</v>
       </c>
-    </row>
-    <row r="13" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="K12">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.75</v>
+      </c>
+      <c r="L12">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="M12" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G13">
         <v>1680</v>
       </c>
@@ -634,8 +731,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.4306640625</v>
       </c>
-    </row>
-    <row r="14" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="K13">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.65625</v>
+      </c>
+      <c r="L13">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.65625</v>
+      </c>
+      <c r="M13" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G14">
         <v>1600</v>
       </c>
@@ -650,8 +759,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.46875</v>
       </c>
-    </row>
-    <row r="15" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.625</v>
+      </c>
+      <c r="L14">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.75</v>
+      </c>
+      <c r="M14" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G15">
         <v>1600</v>
       </c>
@@ -666,8 +787,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.390625</v>
       </c>
-    </row>
-    <row r="16" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.625</v>
+      </c>
+      <c r="L15">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.625</v>
+      </c>
+      <c r="M15" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G16">
         <v>1280</v>
       </c>
@@ -682,8 +815,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.32</v>
       </c>
-    </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.5</v>
+      </c>
+      <c r="L16">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.64</v>
+      </c>
+      <c r="M16" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="7:13" x14ac:dyDescent="0.25">
       <c r="G17">
         <v>1280</v>
       </c>
@@ -698,8 +843,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.25</v>
       </c>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="K17">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.5</v>
+      </c>
+      <c r="L17">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.5</v>
+      </c>
+      <c r="M17" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="7:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="G18">
         <v>1280</v>
       </c>
@@ -714,8 +871,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.22500000000000001</v>
       </c>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="K18">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.5</v>
+      </c>
+      <c r="L18">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.45</v>
+      </c>
+      <c r="M18" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="7:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="G19">
         <v>1024</v>
       </c>
@@ -730,8 +899,20 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.192</v>
       </c>
-    </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.4</v>
+      </c>
+      <c r="L19">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.48</v>
+      </c>
+      <c r="M19" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="7:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="G20">
         <v>800</v>
       </c>
@@ -746,12 +927,30 @@
         <f>(Table1[[#This Row],[Hor]]*Table1[[#This Row],[Ver]])/($G$9*$H$9)</f>
         <v>0.1171875</v>
       </c>
+      <c r="K20">
+        <f>Table1[[#This Row],[Hor]]/$G$9</f>
+        <v>0.3125</v>
+      </c>
+      <c r="L20">
+        <f>Table1[[#This Row],[Ver]]/$H$9</f>
+        <v>0.375</v>
+      </c>
+      <c r="M20" t="b">
+        <f>Table1[[#This Row],[Vert]]=Table1[[#This Row],[Hor2]]</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G9:M20">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$M9</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>